<commit_message>
fix(itr): parse the Dividend quarterly break-up past its blank spacer row
The real report has a completely blank spacer row between the "Quaterly
Break - Up" title and the "Particulars" label row; the parser assumed
adjacency, landed on the blank row, and silently produced zero buckets
with no warning. Now scans forward (bounded) for the label row, reads
ALL following series rows (not just the first -- "Dividend u/s 2(22)(f)"
buyback dividend is a second series), and warns loudly when the title is
found but no label row or no buckets result. QuarterlyBucket gains a
`series` field to carry which row each bucket came from.

Also corrects fixture_gen_fa.py to include the spacer row it was
missing, and regenerates the fixture .xlsx from it.
</commit_message>
<xml_diff>
--- a/tests/skill_itr_workbook/fixtures/syn_indmoney_tax_report.xlsx
+++ b/tests/skill_itr_workbook/fixtures/syn_indmoney_tax_report.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LTCG" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="STCG" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F&amp;O" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Intraday" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dividend" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interest" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bonds &amp; SGB" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schedule FA" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schedule FSI" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Form 67" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schedule TR" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="LTCG" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="STCG" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="F&amp;O" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Intraday" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Dividend" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Interest" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Bonds &amp; SGB" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Schedule FA" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Schedule FSI" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Form 67" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Schedule TR" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1231,7 +1231,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A4:N43"/>
+  <dimension ref="A4:N44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="4">
@@ -1371,263 +1371,231 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Particulars</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>1-Apr to 15-Jun</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>16-Jun to 15-Sep</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>16-Sep to 15-Dec</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>16-Dec to 15-Mar</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>16-Mar to 31-Mar</t>
-        </is>
-      </c>
-    </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Dividend Income</t>
+          <t>Particulars</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>2200</v>
-      </c>
-      <c r="D19" t="n">
-        <v>700</v>
-      </c>
-      <c r="E19" t="n">
-        <v>650</v>
-      </c>
-      <c r="F19" t="n">
-        <v>650</v>
+          <t>1-Apr to 15-Jun</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>16-Jun to 15-Sep</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>16-Sep to 15-Dec</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>16-Dec to 15-Mar</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>16-Mar to 31-Mar</t>
+        </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>Dividend Income</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>2200</v>
+      </c>
+      <c r="D20" t="n">
+        <v>700</v>
+      </c>
+      <c r="E20" t="n">
+        <v>650</v>
+      </c>
+      <c r="F20" t="n">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>Dividend u/s 2(22)(f)</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Indian Stocks Dividend</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Name of Stock</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Ex-Date</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Amount (₹)</t>
+          <t>Indian Stocks Dividend</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Name of Stock</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Ex-Date</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Amount (₹)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C25" t="n">
+      <c r="C26" t="n">
         <v>0</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Dividends From US Stocks</t>
-        </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>Dividends From US Stocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
           <t>Name of the company</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>Date Received</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>Exchange Rates (SBI TT Buying Rates)</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="F29" t="inlineStr">
         <is>
           <t>Tax deducted</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
+      <c r="H29" t="inlineStr">
         <is>
           <t>Broker Name</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="D29" t="inlineStr">
+    <row r="30">
+      <c r="D30" t="inlineStr">
         <is>
           <t>US$</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E30" t="inlineStr">
         <is>
           <t>INR</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="F30" t="inlineStr">
         <is>
           <t>US$</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="G30" t="inlineStr">
         <is>
           <t>INR</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>SynCo Beta Inc. Common Stock</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>2025-06-26</t>
-        </is>
-      </c>
-      <c r="C30" t="n">
-        <v>85.09999999999999</v>
-      </c>
-      <c r="D30" t="n">
-        <v>7.73</v>
-      </c>
-      <c r="E30" t="n">
-        <v>2200</v>
-      </c>
-      <c r="F30" t="n">
-        <v>1.93</v>
-      </c>
-      <c r="G30" t="n">
-        <v>380</v>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>SynBroker LLC</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>SynCo Alpha Ltd American Depositary Shares</t>
+          <t>SynCo Beta Inc. Common Stock</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2025-07-10</t>
+          <t>2025-06-26</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>85.7</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="D31" t="n">
-        <v>8.960000000000001</v>
+        <v>7.73</v>
       </c>
       <c r="E31" t="n">
-        <v>700</v>
+        <v>2200</v>
       </c>
       <c r="F31" t="n">
-        <v>0</v>
+        <v>1.93</v>
       </c>
       <c r="G31" t="n">
-        <v>0</v>
+        <v>380</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
@@ -1643,17 +1611,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2025-10-10</t>
+          <t>2025-07-10</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>88</v>
+        <v>85.7</v>
       </c>
       <c r="D32" t="n">
-        <v>7.39</v>
+        <v>8.960000000000001</v>
       </c>
       <c r="E32" t="n">
-        <v>650</v>
+        <v>700</v>
       </c>
       <c r="F32" t="n">
         <v>0</v>
@@ -1670,19 +1638,19 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>SynCo Beta Inc. Common Stock</t>
+          <t>SynCo Alpha Ltd American Depositary Shares</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2025-12-24</t>
+          <t>2025-10-10</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D33" t="n">
-        <v>7.3</v>
+        <v>7.39</v>
       </c>
       <c r="E33" t="n">
         <v>650</v>
@@ -1702,57 +1670,89 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>SynCo Beta Inc. Common Stock</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2025-12-24</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>89</v>
+      </c>
+      <c r="D34" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="E34" t="n">
+        <v>650</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>SynBroker LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="E34" t="n">
+      <c r="E35" t="n">
         <v>4200</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Disclaimer:-</t>
-        </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>1. This statement has been prepared on a best-effort basis using trade and account information available at the time of report generation.</t>
+          <t>Disclaimer:-</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>4. The tax document is prepared as per the US timezone. So, the numbers presented in this statement may not be equal to other statements which are prepared as per Indian timezone.</t>
+          <t>1. This statement has been prepared on a best-effort basis using trade and account information available at the time of report generation.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>6. Corporate Actions covered in data/report are limited to only Stock Splits and Reverse Stock Splits</t>
+          <t>4. The tax document is prepared as per the US timezone. So, the numbers presented in this statement may not be equal to other statements which are prepared as per Indian timezone.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>7. SBI TT Buy Rate have been used for conversion from USD to INR.</t>
+          <t>6. Corporate Actions covered in data/report are limited to only Stock Splits and Reverse Stock Splits</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>9. The Peak Value and Closing Value of delisted stock will not be included in the reporting.</t>
+          <t>7. SBI TT Buy Rate have been used for conversion from USD to INR.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
+        <is>
+          <t>9. The Peak Value and Closing Value of delisted stock will not be included in the reporting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
         <is>
           <t>16. This tax report excludes INDglobal dividends as they are credited directly to your bank. Please add these manually when filing your return.</t>
         </is>
@@ -1762,13 +1762,13 @@
   <mergeCells count="9">
     <mergeCell ref="A40:N40"/>
     <mergeCell ref="A39:N39"/>
+    <mergeCell ref="F29:G29"/>
     <mergeCell ref="A38:N38"/>
-    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="A43:N43"/>
     <mergeCell ref="A41:N41"/>
-    <mergeCell ref="F28:G28"/>
-    <mergeCell ref="A43:N43"/>
     <mergeCell ref="A42:N42"/>
-    <mergeCell ref="A37:N37"/>
+    <mergeCell ref="A44:N44"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>